<commit_message>
fixing multiple report issues and added grouping functionality
</commit_message>
<xml_diff>
--- a/templates/export/ignition.xlsx
+++ b/templates/export/ignition.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\brnhd\Development\traccar\templates\export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C25A64C-75AA-4F4A-A73E-3C70B7CC8499}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF1E1569-3923-4F34-8EB9-28946897079B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="12645" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ignition" sheetId="1" r:id="rId1"/>
@@ -98,9 +98,6 @@
     <t>${item.geofence}</t>
   </si>
   <si>
-    <t>${item.duration/86400000.0}</t>
-  </si>
-  <si>
     <t>${distanceUnit.equals("mi") ? "".format("%.1f mi", item.distance * 0.000621371) : distanceUnit.equals("nmi") ? "".format("%.1f nmi", item.distance * 0.000539957) : "".format("%.1f km", item.distance * 0.001)}</t>
   </si>
   <si>
@@ -114,6 +111,9 @@
   </si>
   <si>
     <t>${item.endTimeString}</t>
+  </si>
+  <si>
+    <t>${item.engineHours}</t>
   </si>
 </sst>
 </file>
@@ -669,6 +669,114 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>133350</xdr:colOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="6" name="AutoShape 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5E1402EB-113E-7B8F-020D-C114F9C2FF48}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="9525000" cy="9525000"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>133350</xdr:colOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="7" name="AutoShape 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{578A55B2-FF61-F090-4C4B-8CA0704E87BA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="9525000" cy="9525000"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1031,10 +1139,10 @@
       </c>
       <c r="B4" s="5"/>
       <c r="C4" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:1024" x14ac:dyDescent="0.25">
@@ -1078,16 +1186,16 @@
         <v>10</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E7" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="F7" s="12" t="s">
-        <v>16</v>
-      </c>
       <c r="G7" s="10" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="AMF7"/>
       <c r="AMG7"/>

</xml_diff>